<commit_message>
Output Function, Wind, and Demand Adjustments
</commit_message>
<xml_diff>
--- a/Data/Battery.xlsx
+++ b/Data/Battery.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emirsener/Desktop/Campus-Application/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5567B94A-ED43-AE44-BB09-67F12E8BB2DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0935ECE1-133C-D744-9761-9C6F07D23BBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{EDF38AB8-B67A-6545-84A8-C231FAB8949A}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{EDF38AB8-B67A-6545-84A8-C231FAB8949A}"/>
   </bookViews>
   <sheets>
     <sheet name="Initial values" sheetId="7" r:id="rId1"/>
@@ -507,7 +507,7 @@
         <v>12</v>
       </c>
       <c r="B4">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -578,7 +578,7 @@
         <v>21</v>
       </c>
       <c r="B12">
-        <v>6.1000000000000004E-3</v>
+        <v>8.6999999999999994E-3</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>